<commit_message>
chore(data): update Params.xlsx from RH app (Vercel)
</commit_message>
<xml_diff>
--- a/Excel/Params.xlsx
+++ b/Excel/Params.xlsx
@@ -135,10 +135,10 @@
         <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¦ÃÂ¸ÃÂ¸ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯ Light"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ§ÃÂ­ÃÂÃÂ§ÃÂºÃÂ¿ Light"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¦ÃÂÃÂ¸ÃÂÃÂ¸ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯ Light"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ§ÃÂÃÂ­ÃÂÃÂÃÂÃÂ§ÃÂÃÂºÃÂÃÂ¿ Light"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -187,10 +187,10 @@
         <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¦ÃÂ¸ÃÂ¸ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ§ÃÂ­ÃÂÃÂ§ÃÂºÃÂ¿"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¦ÃÂÃÂ¸ÃÂÃÂ¸ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ§ÃÂÃÂ­ÃÂÃÂÃÂÃÂ§ÃÂÃÂºÃÂÃÂ¿"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -790,9 +790,6 @@
       <c r="G3" s="3" t="str">
         <v>[{"menuId":"employes.liste","label":"Liste employés","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"employes.check-documents","label":"Check documents","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"employes.heures","label":"Heures supplémentaires","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"employes.heures.dept","label":"Heures sup. — Département (planning &amp; OT de son département — Modifier = éditer le planning)","actions":{"view":true,"create":true,"edit":true,"delete":true,"export":true}},{"menuId":"employes.heures.all","label":"Heures sup. — Tous départements (planning &amp; OT)","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"employes.heures.import","label":"Heures sup. — Import OT (menu contextuel carte semaine)","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"employes.heures.compilation","label":"Heures sup. — Compilation &amp; politique","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"project.dashboard","label":"Dashboard","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"project.projects","label":"Projects","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"project.expenses","label":"Expenses details","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"travel.etablir","label":"Établir","actions":{"view":true,"create":true,"edit":true,"delete":true,"export":true}},{"menuId":"travel.historique","label":"Historique des voyages","actions":{"view":true,"create":true,"edit":true,"delete":true,"export":true}},{"menuId":"sante","label":"Santé","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"charroi","label":"Charroi automobile","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"settings.departements","label":"Départements","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"settings.centres","label":"Centre de coût","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"settings.utilisateurs","label":"Utilisateurs","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}},{"menuId":"settings.permissions","label":"Permissions","actions":{"view":false,"create":false,"edit":false,"delete":false,"export":false}}]</v>
       </c>
-      <c r="H3" s="3" t="str">
-        <v>{"matricule":"70000049","nom":"Pongo Pongo Charles","departement":"Lab","grade":"D2","jobTitle":"Quality Assurance Manager","localisation":""}</v>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>